<commit_message>
큰 범프 R 로직 정정: 158µm gold를 R0.4→0.77(N58)로 완화
'큰 범프는 R을 높여도 N이 충분'을 명확히 반영. R=√p·D/N이라 D↑→R↑.

- 158µm gold를 R0.4(N112,과잉) → R0.77(N58) 로 완화
  → 158µm R값이 전부 0.77/1.5/3.0 으로 '큰 범프=높은 R' 직관과 일치
  운영 R은 1.5(N30) 유지
- 설계_설명에 R–N–범프크기 관계 섹션 추가:
  N_target 넘으면 시간낭비, 최적 R=N_target 주는 가장 높은 R,
  gold(최저 R)는 기준 truth 앵커일 뿐 운영값 아님
- 55런·35런 동일 반영

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEDPo1aa2m4Ui6JuqiXEbY
</commit_message>
<xml_diff>
--- a/계산모델_엑셀/공정모델링_실험런시트_35런.xlsx
+++ b/계산모델_엑셀/공정모델링_실험런시트_35런.xlsx
@@ -520,14 +520,14 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>■ 장비 제약: R 최소 = 0.2 µm/px  ★신규 반영</t>
+          <t>■ R–N–범프크기 관계 (중요)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>N = 0.283·PD직경 / R. R을 0.2 밑으로 못 내리므로 자재별 '가장 정밀한 N'에 상한이 생김: · 26µm → R0.2에서 N=37이 최대(픽셀오차 5.4%). 더 정밀 불가 → 26µm의 gold=R0.2(N37)이고 R로 속도 벌 여지 거의 없음(R은 0.2에 사실상 고정, 시간단축은 shot수·Frame으로). · 158µm → R0.2에서 N=223로 과잉 → R을 1.5(N30)까지 키워 속도 확보. R 자유도 큼. 결론: 작은 범프일수록 R 자유도가 없다.</t>
+          <t>N = 0.283·PD직경 / R (N=void가 담기는 픽셀 수). 같은 N을 얻는 R = 0.283·D/N → 범프가 클수록 R을 높여도 됨. 'N 클수록 검출 유리'는 맞지만 N_target(~29) 넘으면 판정 오차는 이미 예산 안이라 그 이상은 시간낭비(시간∝1/R²). 따라서 최적 R = N_target을 주는 '가장 높은(거친) R'. 큰 범프일수록 이 값이 높다.</t>
         </is>
       </c>
     </row>
@@ -535,60 +535,22 @@
     <row r="15"/>
     <row r="16"/>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>■ 각 독립변수의 void 측정 메커니즘</t>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>■ 장비 제약 R≥0.2 + 자재별 R (운영값)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>kV</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>대비→경계 이동→void면적 bias. 측정직경(=분모)도 이동시켜 void%에 이중작용.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>픽셀화 오차=2/N. 단 R≥0.2 하한 → 26µm는 N≤37로 제한.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>두꺼운 범프 내부 광자부족→노이즈 void·경계 흔들림. 얇은 범프 둔감.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>랜덤 노이즈 평균화→반복 σ. 시간 정비례.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>· 26µm: R0.2에서 N=37이 최대(픽셀오차5.4%). R 자유도 거의 없음(0.2 고정) → 시간단축은 shot수·Frame. · 158µm: 운영 R=1.5(N30)로 높음. R스윕 최저점 gold(R0.77·N58)은 '기준 truth'용 앵커일 뿐 운영값 아님 (큰 범프는 R 높여도 N 충분). → 작은 범프일수록 R 자유도가 없다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
@@ -599,7 +561,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>교호작용→OFAT 불가. [주효과 스윕+의심 교호작용 2×2+같은범프 반복(σ)]. ε=10% 총예산 (2/N)²+(2σ)²≤10² → N_target≈29(단 26µm은 R하한 탓에 N37 고정)·σ≤3.5%. Ground truth 없어 자기참조(gold)+재현성.</t>
+          <t>교호작용→OFAT 불가. [주효과 스윕+의심 교호작용 2×2+같은범프 반복(σ)]. ε=10% 총예산 (2/N)²+(2σ)²≤10² → N_target≈29(26µm은 R하한 탓 N37)·σ≤3.5%. Ground truth 없어 자기참조(gold)+재현성.</t>
         </is>
       </c>
     </row>
@@ -621,17 +583,15 @@
     </row>
     <row r="31"/>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="12">
     <mergeCell ref="A8:H10"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A12:H12"/>
-    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A25:H27"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="A19:H22"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B20:H20"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="A30:H31"/>
     <mergeCell ref="B5:H5"/>
@@ -680,14 +640,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>직경 다이얼(kV)·void 픽셀화(R). R최소행=gold → 그 void%를 N열에. 26µm gold=R0.2(N37,장비하한) / 158µm gold=R0.4(N112). 고정 F32·W4.</t>
+          <t>직경 다이얼(kV)·void 픽셀화(R). gold(최정밀행)=기준 truth 앵커. 26µm gold=R0.2(N37,장비하한) / 158µm gold=R0.77(N58). 고정 F32·W4.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>D(C열)=PD직경(독립·참값) / 측정직경(J열)=검사결과(종속) / void%(M열)=장비 출력(측정면적 기준) / R≥0.2.</t>
+          <t>D(C열)=PD직경(독립·참값) / 측정직경(J열)=검사결과(종속) / void%(M열)=장비출력(측정면적) / R≥0.2 · 큰 범프일수록 R↑.</t>
         </is>
       </c>
     </row>
@@ -903,7 +863,7 @@
         <v>58.5</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4</v>
+        <v>0.77</v>
       </c>
       <c r="F8">
         <f>IFERROR(ROUND(C8*0.2828/E8,0),"")</f>
@@ -954,7 +914,7 @@
         <v>62.5</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4</v>
+        <v>0.77</v>
       </c>
       <c r="F9">
         <f>IFERROR(ROUND(C9*0.2828/E9,0),"")</f>
@@ -1158,7 +1118,7 @@
         <v>60.5</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4</v>
+        <v>0.77</v>
       </c>
       <c r="F13">
         <f>IFERROR(ROUND(C13*0.2828/E13,0),"")</f>
@@ -1187,7 +1147,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>N≈112 =gold</t>
+          <t>N≈58 =gold(기준앵커)</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1309,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>D(C열)=PD직경(독립·참값) / 측정직경(J열)=검사결과(종속) / void%(M열)=장비 출력(측정면적 기준) / R≥0.2.</t>
+          <t>D(C열)=PD직경(독립·참값) / 측정직경(J열)=검사결과(종속) / void%(M열)=장비출력(측정면적) / R≥0.2 · 큰 범프일수록 R↑.</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2061,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>D(C열)=PD직경(독립·참값) / 측정직경(J열)=검사결과(종속) / void%(M열)=장비 출력(측정면적 기준) / R≥0.2.</t>
+          <t>D(C열)=PD직경(독립·참값) / 측정직경(J열)=검사결과(종속) / void%(M열)=장비출력(측정면적) / R≥0.2 · 큰 범프일수록 R↑.</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2570,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>D(C열)=PD직경(독립·참값) / 측정직경(J열)=검사결과(종속) / void%(M열)=장비 출력(측정면적 기준) / R≥0.2.</t>
+          <t>D(C열)=PD직경(독립·참값) / 측정직경(J열)=검사결과(종속) / void%(M열)=장비출력(측정면적) / R≥0.2 · 큰 범프일수록 R↑.</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2859,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(모델R)</t>
+          <t>(모델R,높음)</t>
         </is>
       </c>
       <c r="F9">
@@ -2960,7 +2920,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(모델R)</t>
+          <t>(모델R,높음)</t>
         </is>
       </c>
       <c r="F10">
@@ -3013,7 +2973,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(모델R)</t>
+          <t>(모델R,높음)</t>
         </is>
       </c>
       <c r="F11">
@@ -3107,7 +3067,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Phase1 R스윕: gold 대비 |void편차| 7% 넘는 N(≈29). 단 26µm은 R하한으로 N37 고정→R0.2</t>
+          <t>Phase1 R스윕: gold 대비 |void편차| 7% 넘는 N(≈29). 26µm은 R하한→N37 고정(R0.2)</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3158,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>R=max(0.2, D·√p/N_target). 작은 범프는 0.2에 걸림</t>
+          <t>R = max(0.2, D·√p/N_target). 큰 범프일수록 R↑ / 작은 범프는 0.2에 걸림</t>
         </is>
       </c>
     </row>

</xml_diff>